<commit_message>
slot-unlimited-codex story-004：卡表补 6 个器官获得入口（8008/8009/8018/8019/8020/8024），Luban 重生 Tables.cs + GameRes 指针 bump
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/cell/#Card-卡牌.xlsx
+++ b/Configs/GameConfig/Datas/cell/#Card-卡牌.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T31"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1215,16 +1215,16 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>8011</v>
+        <v>8008</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>液泡电容</t>
+          <t>粘液层</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>接入切片：按倍率放大流经的能量。</t>
+          <t>接入切片：给流经的信号打上「油」标记。</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1234,14 +1234,14 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1278,23 +1278,23 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>org_vacuole</t>
+          <t>org_slime</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>8012</v>
+        <v>8009</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>高尔基分流</t>
+          <t>受体</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>接入切片：把能量均分给多条支路。</t>
+          <t>接入切片：给流经的信号打上「催化」标记。</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1304,14 +1304,14 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1348,23 +1348,23 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>org_golgi</t>
+          <t>org_receptor</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>8013</v>
+        <v>8011</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>晶状聚焦</t>
+          <t>液泡电容</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>接入切片：提升伤害的同时必定增加热量。</t>
+          <t>接入切片：按倍率放大流经的能量。</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1418,23 +1418,23 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>org_lens</t>
+          <t>org_vacuole</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>8014</v>
+        <v>8012</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>纺锤散射</t>
+          <t>高尔基分流</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>接入切片：按当前倍率把信号分裂成多份。</t>
+          <t>接入切片：把能量均分给多条支路。</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1488,23 +1488,23 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>org_scatter</t>
+          <t>org_golgi</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>8015</v>
+        <v>8013</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>膨胀泡</t>
+          <t>晶状聚焦</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>接入切片：放大弹体尺度。</t>
+          <t>接入切片：提升伤害的同时必定增加热量。</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1558,23 +1558,23 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>org_swell</t>
+          <t>org_lens</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>8016</v>
+        <v>8014</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>鞭毛环</t>
+          <t>纺锤散射</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>接入切片：让弹体沿圆周轨迹运动。</t>
+          <t>接入切片：按当前倍率把信号分裂成多份。</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1628,23 +1628,23 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>org_flagella</t>
+          <t>org_scatter</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>8017</v>
+        <v>8015</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>溶酶爆</t>
+          <t>膨胀泡</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>接入切片：命中即触发范围爆炸。</t>
+          <t>接入切片：放大弹体尺度。</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1698,23 +1698,23 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>org_lyso</t>
+          <t>org_swell</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>8021</v>
+        <v>8016</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>散热褶</t>
+          <t>鞭毛环</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>接入切片：压低链路热量，避免过载跳闸。</t>
+          <t>接入切片：让弹体沿圆周轨迹运动。</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1724,14 +1724,14 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
         <v>2</v>
-      </c>
-      <c r="H18" t="n">
-        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1768,23 +1768,23 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>org_radiator</t>
+          <t>org_flagella</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>8022</v>
+        <v>8017</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>热休克闸</t>
+          <t>溶酶爆</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>接入切片：能量超过安全上限时强制夹住，防止溢出。</t>
+          <t>接入切片：命中即触发范围爆炸。</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1794,14 +1794,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
         <v>2</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1838,23 +1838,23 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>org_breaker</t>
+          <t>org_lyso</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>8023</v>
+        <v>8018</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>突触反馈</t>
+          <t>囊泡汇流</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>接入切片：命中后把部分能量反馈回自身链路。</t>
+          <t>接入切片：把入流能量夹到带宽上限，超出部分折半转为热量。</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1864,14 +1864,14 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
         <v>2</v>
-      </c>
-      <c r="H20" t="n">
-        <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1908,23 +1908,23 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>org_synapse</t>
+          <t>org_merge</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="n">
-        <v>8101</v>
+        <v>8019</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>燃律</t>
+          <t>单向阀</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>全局法则：命中额外附带燃烧强度。</t>
+          <t>接入切片：强化沿链方向流动的能量。</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1934,14 +1934,14 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1973,28 +1973,28 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>gene_pyro</t>
+          <t>org_valve</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>8102</v>
+        <v>8020</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>潮律</t>
+          <t>刺突</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>全局法则：命中额外附带潮湿强度。</t>
+          <t>接入切片：受击时反弹固定伤害。</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2004,14 +2004,14 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2043,28 +2043,28 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>gene_tide</t>
+          <t>org_spine</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>8103</v>
+        <v>8021</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>雷律</t>
+          <t>散热褶</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>全局法则：命中额外附带感电强度。</t>
+          <t>接入切片：压低链路热量，避免过载跳闸。</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2074,14 +2074,14 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2113,28 +2113,28 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>gene_volt</t>
+          <t>org_radiator</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>8104</v>
+        <v>8022</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>共相</t>
+          <t>热休克闸</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>全局法则：与友方共享承伤状态。</t>
+          <t>接入切片：能量超过安全上限时强制夹住，防止溢出。</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2144,14 +2144,14 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2183,28 +2183,28 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>gene_share</t>
+          <t>org_breaker</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>8111</v>
+        <v>8023</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>双倍表达</t>
+          <t>突触反馈</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>全局法则：大幅提升伤害倍率（过载许可）。</t>
+          <t>接入切片：命中后把部分能量反馈回自身链路。</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2214,14 +2214,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2253,28 +2253,28 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>gene_double</t>
+          <t>org_synapse</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>8112</v>
+        <v>8024</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>延偿</t>
+          <t>过滤管</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>全局法则：伤害结算延后，多次叠加取最大延迟。</t>
+          <t>接入切片：只放行带指定标记的能量，未命中的按比例折损。</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2284,14 +2284,14 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2323,28 +2323,28 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>gene_delay</t>
+          <t>org_filter</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>8113</v>
+        <v>8101</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>寡兵</t>
+          <t>燃律</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>全局法则：单位越少，输出曲线越陡。</t>
+          <t>全局法则：命中额外附带燃烧强度。</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2354,14 +2354,14 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2398,23 +2398,23 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>gene_swarm</t>
+          <t>gene_pyro</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>8114</v>
+        <v>8102</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>哑火</t>
+          <t>潮律</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>全局法则：禁用远程输出，并强制关闭反射。</t>
+          <t>全局法则：命中额外附带潮湿强度。</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2424,14 +2424,14 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2468,23 +2468,23 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>gene_mute</t>
+          <t>gene_tide</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>8121</v>
+        <v>8103</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>镜界</t>
+          <t>雷律</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>全局法则：开启完全反射（与哑火冲突，后应用者生效）。</t>
+          <t>全局法则：命中额外附带感电强度。</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2494,14 +2494,14 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2538,23 +2538,23 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>gene_mirror</t>
+          <t>gene_volt</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>8122</v>
+        <v>8104</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>血债</t>
+          <t>共相</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>全局法则：造成的伤害部分转化为治疗。</t>
+          <t>全局法则：与友方共享承伤状态。</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2564,14 +2564,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2608,23 +2608,23 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>gene_blood</t>
+          <t>gene_share</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>8123</v>
+        <v>8111</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>绝境</t>
+          <t>双倍表达</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>全局法则：残血状态下承受伤害打折。</t>
+          <t>全局法则：大幅提升伤害倍率（过载许可）。</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2634,14 +2634,14 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="n">
         <v>2</v>
-      </c>
-      <c r="H31" t="n">
-        <v>1</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2677,6 +2677,426 @@
         </is>
       </c>
       <c r="T31" t="inlineStr">
+        <is>
+          <t>gene_double</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="n">
+        <v>8112</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>延偿</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>全局法则：伤害结算延后，多次叠加取最大延迟。</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="n">
+        <v>2</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>gene_delay</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+      <c r="B33" t="n">
+        <v>8113</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>寡兵</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>全局法则：单位越少，输出曲线越陡。</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>gene_swarm</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" t="n">
+        <v>8114</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>哑火</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>全局法则：禁用远程输出，并强制关闭反射。</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>gene_mute</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="n">
+        <v>8121</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>镜界</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>全局法则：开启完全反射（与哑火冲突，后应用者生效）。</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>gene_mirror</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="n">
+        <v>8122</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>血债</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>全局法则：造成的伤害部分转化为治疗。</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>gene_blood</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="n">
+        <v>8123</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>绝境</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>全局法则：残血状态下承受伤害打折。</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
         <is>
           <t>gene_edge</t>
         </is>

</xml_diff>

<commit_message>
combat-identity-rework story-010: 抽卡池同步 24+24 目录
沙盒器官列表（BattleSandboxUIToolkit/CellDebugHud）漏过滤 AttackMethod，
退役修饰（含高尔基分流 org_golgi）仍可选中，顺藤查出真正的抽卡池
（Luban TbCard）从未同步 combat-identity-rework 的器官/基因退役迁移，
被 CellLubanLoader 的运行时过滤静默挡住大半内容。

- BattleSandboxUIToolkit.cs / CellDebugHud.cs：器官列表加 AttackMethod 过滤
- ShopSystem.ShopOrganelleIds：org_mito/org_lens 废件换成 org_cilia/org_lensbeam
- carddata.py 按 CATALOG.md §C 映射全表重写，Luban 重生 Tables.cs/cell_tbcard.bytes：
  24 基因全覆盖（6→24），24 攻击器官 11 条可抽（4→11）
- CellLubanLoader.cs：更新已过时的"表改不动"注释，过滤逻辑保留作兜底安全网

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/cell/#Card-卡牌.xlsx
+++ b/Configs/GameConfig/Datas/cell/#Card-卡牌.xlsx
@@ -725,16 +725,16 @@
     <row r="4">
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="n">
-        <v>8001</v>
+        <v>8003</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>线粒体</t>
+          <t>分泌喷射器</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>接入切片：持续产出基础能量，是产链的起点。</t>
+          <t>攻击方式：朝瞄准方向射出代谢弹。</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -788,23 +788,23 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>org_mito</t>
+          <t>org_emitter</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="n">
-        <v>8002</v>
+        <v>8004</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>叶绿体</t>
+          <t>纤毛刺</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>接入切片：另一种能量起点，效果与线粒体同源。</t>
+          <t>攻击方式：身前短锥挥刺。</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -858,23 +858,23 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>org_chloro</t>
+          <t>org_cilia</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="n">
-        <v>8003</v>
+        <v>8013</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>分泌喷射器</t>
+          <t>晶状束</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>接入切片：把链路能量折算成一次攻击输出。</t>
+          <t>攻击方式：一条持续细束，扫过伤害。</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -884,14 +884,14 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -928,23 +928,23 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>org_emitter</t>
+          <t>org_lensbeam</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="n">
-        <v>8004</v>
+        <v>8020</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>纤毛刺</t>
+          <t>刺突</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>接入切片：另一种输出终端，效果与分泌喷射器同源。</t>
+          <t>攻击方式：被碰到或挨打时反刺，不靠主动开火。</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -954,14 +954,14 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -998,23 +998,23 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>org_cilia</t>
+          <t>org_spine</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="n">
-        <v>8005</v>
+        <v>8025</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>过氧化物酶</t>
+          <t>吞噬体</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>接入切片：给流经的信号打上「燃」标记。</t>
+          <t>攻击方式：接触到体积小于自身的目标时直接吞噬消灭；不主动开火。</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1068,23 +1068,23 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>org_perox</t>
+          <t>org_phago</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="n">
-        <v>8006</v>
+        <v>8001</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>水合泡</t>
+          <t>酶雾腺</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>接入切片：给流经的信号打上「潮」标记。</t>
+          <t>攻击方式：把酶雾扔到落点，地面持续腐蚀。</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1138,23 +1138,23 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>org_aqua</t>
+          <t>org_enzyme</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="n">
-        <v>8007</v>
+        <v>8002</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>离子泵</t>
+          <t>趋化索</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>接入切片：给流经的信号打上「电」标记。</t>
+          <t>攻击方式：弹自己会拐去最近敌人。</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1208,23 +1208,23 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>org_ion</t>
+          <t>org_taxis</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>8008</v>
+        <v>8018</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>粘液层</t>
+          <t>渗透压场</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>接入切片：给流经的信号打上「油」标记。</t>
+          <t>攻击方式：身体周围一圈压差，进圈就伤。</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1234,14 +1234,14 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1278,23 +1278,23 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>org_slime</t>
+          <t>org_osmotic</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>8009</v>
+        <v>8019</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>受体</t>
+          <t>纤毛环带</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>接入切片：给流经的信号打上「催化」标记。</t>
+          <t>攻击方式：两枚体绕身旋转打人（圣经感）。</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1304,14 +1304,14 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1348,23 +1348,23 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>org_receptor</t>
+          <t>org_orbitcilia</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>8011</v>
+        <v>8022</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>液泡电容</t>
+          <t>胞吐霰</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>接入切片：按倍率放大流经的能量。</t>
+          <t>攻击方式：近距扇形多弹。</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1418,23 +1418,23 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>org_vacuole</t>
+          <t>org_shotgun</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>8012</v>
+        <v>8024</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>高尔基分流</t>
+          <t>放电突触</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>接入切片：把能量均分给多条支路。</t>
+          <t>攻击方式：跳到附近下一只。</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1444,14 +1444,14 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1488,23 +1488,23 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>org_golgi</t>
+          <t>org_synapsearc</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>8013</v>
+        <v>8005</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>晶状聚焦</t>
+          <t>趋化导引</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>接入切片：提升伤害的同时必定增加热量。</t>
+          <t>需要器官。改装：攻击会拐向敌人。</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1514,14 +1514,14 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1553,28 +1553,28 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>org_lens</t>
+          <t>gene_taxis</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>8014</v>
+        <v>8006</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>纺锤散射</t>
+          <t>微管贯穿</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>接入切片：按当前倍率把信号分裂成多份。</t>
+          <t>需要器官。改装：穿过目标继续飞。</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1584,14 +1584,14 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1623,28 +1623,28 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>org_scatter</t>
+          <t>gene_tubule</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>8015</v>
+        <v>8007</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>膨胀泡</t>
+          <t>弹性壁</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>接入切片：放大弹体尺度。</t>
+          <t>需要器官。改装：撞边或撞敌会弹。</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1654,14 +1654,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1693,28 +1693,28 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>org_swell</t>
+          <t>gene_elastic</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>8016</v>
+        <v>8008</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>鞭毛环</t>
+          <t>粘液拖尾</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>接入切片：让弹体沿圆周轨迹运动。</t>
+          <t>需要器官。改装：路径减速并伤。</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1724,14 +1724,14 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1763,28 +1763,28 @@
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>org_flagella</t>
+          <t>gene_slime</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>8017</v>
+        <v>8009</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>溶酶爆</t>
+          <t>受体记忆</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>接入切片：命中即触发范围爆炸。</t>
+          <t>需要器官。改装：打过的敌人会被记住，后续更会追它。</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1794,14 +1794,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1833,28 +1833,28 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>org_lyso</t>
+          <t>gene_receptor</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>8018</v>
+        <v>8101</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>囊泡汇流</t>
+          <t>燃径</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>接入切片：把入流能量夹到带宽上限，超出部分折半转为热量。</t>
+          <t>需要器官。改装：飞过或命中铺火径，不是只挂燃烧数字。</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1864,14 +1864,14 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1903,28 +1903,28 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>org_merge</t>
+          <t>gene_pyro</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="n">
-        <v>8019</v>
+        <v>8102</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>单向阀</t>
+          <t>潮洼</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>接入切片：强化沿链方向流动的能量。</t>
+          <t>需要器官。改装：留下水洼；水洼让雷跳、让火变蒸汽。</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1934,14 +1934,14 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1973,28 +1973,28 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>org_valve</t>
+          <t>gene_tide</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>8020</v>
+        <v>8103</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>刺突</t>
+          <t>雷桥</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>接入切片：受击时反弹固定伤害。</t>
+          <t>需要器官。改装：优先沿湿面/水洼跳。</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2004,14 +2004,14 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -2043,28 +2043,28 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>org_spine</t>
+          <t>gene_volt</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>8021</v>
+        <v>8104</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>散热褶</t>
+          <t>回旋外壳</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>接入切片：压低链路热量，避免过载跳闸。</t>
+          <t>需要器官。改装：打出的东西会飞回来。</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2074,14 +2074,14 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2113,28 +2113,28 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>org_radiator</t>
+          <t>gene_return</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>8022</v>
+        <v>8011</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>热休克闸</t>
+          <t>蓄能液泡</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>接入切片：能量超过安全上限时强制夹住，防止溢出。</t>
+          <t>需要器官。改装：少打几下，下一发更肥。</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2144,14 +2144,14 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="n">
         <v>2</v>
-      </c>
-      <c r="H24" t="n">
-        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2183,28 +2183,28 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>org_breaker</t>
+          <t>gene_vacuole</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>8023</v>
+        <v>8012</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>突触反馈</t>
+          <t>分流芽</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>接入切片：命中后把部分能量反馈回自身链路。</t>
+          <t>需要器官。改装：半路或出手时分叉。</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2214,14 +2214,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="n">
         <v>2</v>
-      </c>
-      <c r="H25" t="n">
-        <v>1</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2253,28 +2253,28 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>org_synapse</t>
+          <t>gene_golgi</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>8024</v>
+        <v>8014</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>过滤管</t>
+          <t>纺锤分裂</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>接入切片：只放行带指定标记的能量，未命中的按比例折损。</t>
+          <t>需要器官。改装：一次打出更多、更散。</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2284,14 +2284,14 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="n">
         <v>2</v>
-      </c>
-      <c r="H26" t="n">
-        <v>1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2323,28 +2323,28 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>org_filter</t>
+          <t>gene_spindle</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>8025</v>
+        <v>8015</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>吞噬体</t>
+          <t>膨胀泡</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>接入切片：接触到体积小于自身的目标时直接吞噬消灭，不主动开火。</t>
+          <t>需要器官。改装：体变大、圈变大、坑变大。</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2354,14 +2354,14 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2393,28 +2393,28 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Organelle</t>
+          <t>Gene</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>org_phago</t>
+          <t>gene_swell</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>8101</v>
+        <v>8016</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>燃律</t>
+          <t>鞭毛绕</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>全局法则：命中额外附带燃烧强度。</t>
+          <t>需要器官。改装：攻击绕圈飞/绕着你转。</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2424,14 +2424,14 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2468,23 +2468,23 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>gene_pyro</t>
+          <t>gene_flagella</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>8102</v>
+        <v>8017</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>潮律</t>
+          <t>溶酶壳</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>全局法则：命中额外附带潮湿强度。</t>
+          <t>需要器官。改装：命中再爆一圈。</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2494,14 +2494,14 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2538,23 +2538,23 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>gene_tide</t>
+          <t>gene_lyso</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>8103</v>
+        <v>8113</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>雷律</t>
+          <t>群体感应</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>全局法则：命中额外附带感电强度。</t>
+          <t>需要器官。改装：你的召唤物学会这件器官的打法。</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2564,14 +2564,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2608,23 +2608,23 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>gene_volt</t>
+          <t>gene_swarm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>8104</v>
+        <v>8111</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>共相</t>
+          <t>残影</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>全局法则：与友方共享承伤状态。</t>
+          <t>需要器官。改装：命中点稍后自己再打一次。</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2634,14 +2634,14 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2678,23 +2678,23 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>gene_share</t>
+          <t>gene_echo</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>8111</v>
+        <v>8112</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>双倍表达</t>
+          <t>吸引素</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>全局法则：大幅提升伤害倍率（过载许可）。</t>
+          <t>需要器官。改装：把敌人往弹/圈/坑里吸。</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2748,23 +2748,23 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>gene_double</t>
+          <t>gene_pull</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>8112</v>
+        <v>8114</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>延偿</t>
+          <t>绽放</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>全局法则：伤害结算延后，多次叠加取最大延迟。</t>
+          <t>需要器官。改装：命中裂成小弹。</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2818,23 +2818,23 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>gene_delay</t>
+          <t>gene_split</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>8113</v>
+        <v>8021</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>寡兵</t>
+          <t>热激褶</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>全局法则：单位越少，输出曲线越陡。</t>
+          <t>需要器官。改装：过热时爆一圈，而不是「默默降温」。</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2844,14 +2844,14 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2888,23 +2888,23 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>gene_swarm</t>
+          <t>gene_heatshock</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>8114</v>
+        <v>8023</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>哑火</t>
+          <t>突触连发</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>全局法则：禁用远程输出，并强制关闭反射。</t>
+          <t>需要器官。改装：命中立刻再挤一发。</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2914,14 +2914,14 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>gene_mute</t>
+          <t>gene_synapse</t>
         </is>
       </c>
     </row>
@@ -2969,12 +2969,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>镜界</t>
+          <t>镜面</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>全局法则：开启完全反射（与哑火冲突，后应用者生效）。</t>
+          <t>需要器官。改装：弹会反弹；近战则弹开敌人的弹。</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3039,12 +3039,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>血债</t>
+          <t>血珠</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>全局法则：造成的伤害部分转化为治疗。</t>
+          <t>需要器官。改装：打出的伤害溅出血珠飞回治疗。</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3109,12 +3109,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>绝境</t>
+          <t>凋亡信号</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>全局法则：残血状态下承受伤害打折。</t>
+          <t>需要器官。改装：残血敌人被打中会爆开，不是冻死。</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>gene_edge</t>
+          <t>gene_apoptosis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
organ-gene-rebalance-v3 story-007：抽卡池 carddata.py 迁移到 13 器官+42 基因全覆盖
按 CATALOG-v3 §C 把指向已退役 org_taxis/org_shotgun/org_synapsearc 的 3 张卡改指向迁移
基因（gene_taxis/gene_fan/gene_volt），补 5 张此前无卡的攻击器官（org_wave/pseudopod/
drill/bud/mycelium）与 17 张此前无卡的新增基因，凑满 13 器官 + 42 基因全部可抽（57 张
Card）。carddata.py 源码在根仓库 tools/cell_tables/，本仓只提交 gen_all.py 重生的
cell.* xlsx + Luban codegen 后的 GameRes bytes 指针。execute_code 断言：Loaded=True，
UsingFallback=False（真读 Luban 非内置兜底），OrganCardKinds=13/GeneCardKinds=42，
RetiredOrganCardsOnPool 为空。
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/cell/#Card-卡牌.xlsx
+++ b/Configs/GameConfig/Datas/cell/#Card-卡牌.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T38"/>
+  <dimension ref="A1:T60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1145,16 +1145,16 @@
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="n">
-        <v>8002</v>
+        <v>8018</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>趋化索</t>
+          <t>渗透压场</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>攻击方式：弹自己会拐去最近敌人。</t>
+          <t>攻击方式：身体周围一圈压差，进圈就伤。</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1164,14 +1164,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1208,23 +1208,23 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>org_taxis</t>
+          <t>org_osmotic</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="n">
-        <v>8018</v>
+        <v>8019</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>渗透压场</t>
+          <t>纤毛环带</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>攻击方式：身体周围一圈压差，进圈就伤。</t>
+          <t>攻击方式：两枚体绕身旋转打人。</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1278,23 +1278,23 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>org_osmotic</t>
+          <t>org_orbitcilia</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="n">
-        <v>8019</v>
+        <v>8026</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>纤毛环带</t>
+          <t>波形器</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>攻击方式：两枚体绕身旋转打人（圣经感）。</t>
+          <t>攻击方式：朝面向打出可扩散的新月波（合并旧钙波环+胞质浪几何身份）。</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1348,23 +1348,23 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>org_orbitcilia</t>
+          <t>org_wave</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="n">
-        <v>8022</v>
+        <v>8027</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>胞吐霰</t>
+          <t>伪足拍</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>攻击方式：近距扇形多弹。</t>
+          <t>攻击方式：身前宽拍并击退。</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1374,14 +1374,14 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1418,23 +1418,23 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>org_shotgun</t>
+          <t>org_pseudopod</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="n">
-        <v>8024</v>
+        <v>8028</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>放电突触</t>
+          <t>纤毛钻</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>攻击方式：跳到附近下一只。</t>
+          <t>攻击方式：短冲刺，路径上穿刺。</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1444,14 +1444,14 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
         <v>2</v>
-      </c>
-      <c r="H14" t="n">
-        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1488,23 +1488,23 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>org_synapsearc</t>
+          <t>org_drill</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="n">
-        <v>8005</v>
+        <v>8029</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>趋化导引</t>
+          <t>芽殖体</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>需要器官。改装：攻击会拐向敌人。</t>
+          <t>攻击方式：长出跟随的芽体帮你打（吸收旧孢子云/噬菌体召唤语义）。</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1514,14 +1514,14 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1553,28 +1553,28 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>gene_taxis</t>
+          <t>org_bud</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="n">
-        <v>8006</v>
+        <v>8030</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>微管贯穿</t>
+          <t>菌丝锚</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>需要器官。改装：穿过目标继续飞。</t>
+          <t>攻击方式：钉一根菌丝炮台，定点打附近。</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1584,14 +1584,14 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Epic</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1623,28 +1623,28 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Gene</t>
+          <t>Organelle</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>gene_tubule</t>
+          <t>org_mycelium</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="n">
-        <v>8007</v>
+        <v>8005</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>弹性壁</t>
+          <t>趋化导引</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>需要器官。改装：撞边或撞敌会弹。</t>
+          <t>需要器官。改装：攻击会拐向敌人。</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1698,23 +1698,23 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>gene_elastic</t>
+          <t>gene_taxis</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="n">
-        <v>8008</v>
+        <v>8006</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>粘液拖尾</t>
+          <t>微管贯穿</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>需要器官。改装：路径减速并伤。</t>
+          <t>需要器官。改装：穿过目标继续飞。</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1768,23 +1768,23 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>gene_slime</t>
+          <t>gene_tubule</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="n">
-        <v>8009</v>
+        <v>8007</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>受体记忆</t>
+          <t>弹性壁</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>需要器官。改装：打过的敌人会被记住，后续更会追它。</t>
+          <t>需要器官。改装：撞边或撞敌会弹。</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1838,23 +1838,23 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>gene_receptor</t>
+          <t>gene_elastic</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="n">
-        <v>8101</v>
+        <v>8008</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>燃径</t>
+          <t>粘液拖尾</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>需要器官。改装：飞过或命中铺火径，不是只挂燃烧数字。</t>
+          <t>需要器官。改装：路径减速并伤。</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1908,23 +1908,23 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>gene_pyro</t>
+          <t>gene_slime</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="n">
-        <v>8102</v>
+        <v>8009</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>潮洼</t>
+          <t>受体记忆</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>需要器官。改装：留下水洼；水洼让雷跳、让火变蒸汽。</t>
+          <t>需要器官。改装：打过的敌人会被记住，后续更会追它。</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1978,23 +1978,23 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>gene_tide</t>
+          <t>gene_receptor</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="n">
-        <v>8103</v>
+        <v>8101</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>雷桥</t>
+          <t>燃径</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>需要器官。改装：优先沿湿面/水洼跳。</t>
+          <t>需要器官。改装：飞过或命中铺火径，不是只挂燃烧数字。</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2048,23 +2048,23 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>gene_volt</t>
+          <t>gene_pyro</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="n">
-        <v>8104</v>
+        <v>8102</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>回旋外壳</t>
+          <t>潮洼</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>需要器官。改装：打出的东西会飞回来。</t>
+          <t>需要器官。改装：留下水洼；水洼让雷跳、让火变蒸汽。</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2118,23 +2118,23 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>gene_return</t>
+          <t>gene_tide</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="n">
-        <v>8011</v>
+        <v>8103</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>蓄能液泡</t>
+          <t>雷桥</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>需要器官。改装：少打几下，下一发更肥。</t>
+          <t>需要器官。改装：优先沿湿面/水洼跳。</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2144,14 +2144,14 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2188,23 +2188,23 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>gene_vacuole</t>
+          <t>gene_volt</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="n">
-        <v>8012</v>
+        <v>8104</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>分流芽</t>
+          <t>回旋外壳</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>需要器官。改装：半路或出手时分叉。</t>
+          <t>需要器官。改装：打出的东西会飞回来。</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2214,14 +2214,14 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Rare</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2258,23 +2258,23 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>gene_golgi</t>
+          <t>gene_return</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="n">
-        <v>8014</v>
+        <v>8011</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>纺锤分裂</t>
+          <t>蓄能液泡</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>需要器官。改装：一次打出更多、更散。</t>
+          <t>需要器官。改装：少打几下，下一发更肥。</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2328,23 +2328,23 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>gene_spindle</t>
+          <t>gene_vacuole</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="n">
-        <v>8015</v>
+        <v>8012</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>膨胀泡</t>
+          <t>分流芽</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>需要器官。改装：体变大、圈变大、坑变大。</t>
+          <t>需要器官。改装：半路或出手时分叉。</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2398,23 +2398,23 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>gene_swell</t>
+          <t>gene_golgi</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="n">
-        <v>8016</v>
+        <v>8014</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>鞭毛绕</t>
+          <t>纺锤分裂</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>需要器官。改装：攻击绕圈飞/绕着你转。</t>
+          <t>需要器官。改装：一次打出更多、更散。</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2468,23 +2468,23 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>gene_flagella</t>
+          <t>gene_spindle</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="n">
-        <v>8017</v>
+        <v>8015</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>溶酶壳</t>
+          <t>膨胀泡</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>需要器官。改装：命中再爆一圈。</t>
+          <t>需要器官。改装：体变大、圈变大、坑变大。</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2538,23 +2538,23 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>gene_lyso</t>
+          <t>gene_swell</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="n">
-        <v>8113</v>
+        <v>8016</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>群体感应</t>
+          <t>鞭毛绕</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>需要器官。改装：你的召唤物学会这件器官的打法。</t>
+          <t>需要器官。改装：攻击绕圈飞/绕着你转。</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2608,23 +2608,23 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>gene_swarm</t>
+          <t>gene_flagella</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="n">
-        <v>8111</v>
+        <v>8017</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>残影</t>
+          <t>溶酶壳</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>需要器官。改装：命中点稍后自己再打一次。</t>
+          <t>需要器官。改装：命中再爆一圈。</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2678,23 +2678,23 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>gene_echo</t>
+          <t>gene_lyso</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="n">
-        <v>8112</v>
+        <v>8113</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>吸引素</t>
+          <t>群体感应</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>需要器官。改装：把敌人往弹/圈/坑里吸。</t>
+          <t>需要器官。改装：你的召唤物学会这件器官的打法。</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2748,23 +2748,23 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>gene_pull</t>
+          <t>gene_swarm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="n">
-        <v>8114</v>
+        <v>8111</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>绽放</t>
+          <t>残影</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>需要器官。改装：命中裂成小弹。</t>
+          <t>需要器官。改装：命中点稍后自己再打一次。</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2818,23 +2818,23 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>gene_split</t>
+          <t>gene_echo</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="n">
-        <v>8021</v>
+        <v>8112</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>热激褶</t>
+          <t>吸引素</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>需要器官。改装：过热时爆一圈，而不是「默默降温」。</t>
+          <t>需要器官。改装：把敌人往弹/圈/坑里吸。</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -2844,14 +2844,14 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="n">
         <v>2</v>
-      </c>
-      <c r="H34" t="n">
-        <v>1</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2888,23 +2888,23 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>gene_heatshock</t>
+          <t>gene_pull</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="n">
-        <v>8023</v>
+        <v>8114</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>突触连发</t>
+          <t>绽放</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>需要器官。改装：命中立刻再挤一发。</t>
+          <t>需要器官。改装：命中裂成小弹。</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2914,14 +2914,14 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="n">
         <v>2</v>
-      </c>
-      <c r="H35" t="n">
-        <v>1</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2958,23 +2958,23 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>gene_synapse</t>
+          <t>gene_split</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>8121</v>
+        <v>8021</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>镜面</t>
+          <t>热激褶</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>需要器官。改装：弹会反弹；近战则弹开敌人的弹。</t>
+          <t>需要器官。改装：过热时爆一圈，而不是「默默降温」。</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3028,23 +3028,23 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>gene_mirror</t>
+          <t>gene_heatshock</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>8122</v>
+        <v>8023</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>血珠</t>
+          <t>突触连发</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>需要器官。改装：打出的伤害溅出血珠飞回治疗。</t>
+          <t>需要器官。改装：命中立刻再挤一发。</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3098,23 +3098,23 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>gene_blood</t>
+          <t>gene_synapse</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>8123</v>
+        <v>8121</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>凋亡信号</t>
+          <t>镜面</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>需要器官。改装：残血敌人被打中会爆开，不是冻死。</t>
+          <t>需要器官。改装：弹会反弹；近战则弹开敌人的弹。</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3168,7 +3168,1547 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
+          <t>gene_mirror</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="n">
+        <v>8122</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>血珠</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>需要器官。改装：打出的伤害溅出血珠飞回治疗。</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="n">
+        <v>1</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>gene_blood</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="n">
+        <v>8123</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>凋亡信号</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>需要器官。改装：残血敌人被打中会爆开，不是冻死。</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0</v>
+      </c>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
           <t>gene_apoptosis</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="n">
+        <v>8002</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>趋化索（基因）</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>需要器官。改装：攻击会拐向敌人（原趋化索器官迁移基因，CATALOG-v3 §C）。</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>gene_taxis</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="n">
+        <v>8022</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>胞吐霰（基因）</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>需要器官。改装：让扇面变宽或变窄（原胞吐霰器官迁移基因，CATALOG-v3 §C）。</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="n">
+        <v>2</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>gene_fan</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="n">
+        <v>8024</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>放电突触（基因）</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>需要器官。改装：优先沿湿面/水洼跳（原放电突触器官迁移基因，CATALOG-v3 §C）。</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" t="n">
+        <v>1</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>gene_volt</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="n">
+        <v>8124</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>扩散波</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>需要器官。改装：波/圈会随时间越扩越大，不是一下子变大。</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>3</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>gene_ripple</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="n">
+        <v>8125</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>节律</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>需要器官。改装：按固定节拍自己再打一圈。</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0</v>
+      </c>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>gene_rhythm</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="n">
+        <v>8126</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>乱流</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>需要器官。改装：弹道会随机侧偏，飘忽不定。</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>3</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>gene_drift</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="n">
+        <v>8127</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>油膜</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>需要器官。改装：命中处留下油膜，遇火会烧起来。</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>gene_oilfilm</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="n">
+        <v>8128</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>糖膜</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>需要器官。改装：命中处留下糖膜，遇酸会变粘滞。</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>3</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>gene_sugarfilm</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="n">
+        <v>8129</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>涡旋</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>需要器官。改装：边转边把敌人往里吸。</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Common</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>3</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>gene_vortex</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="n">
+        <v>8130</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>酸蚀膜</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>需要器官。改装：落点变成酸坑，持续腐蚀。</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="n">
+        <v>2</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0</v>
+      </c>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>gene_acidfilm</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="n">
+        <v>8131</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>霜膜</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>需要器官。改装：命中处结一层霜（不致死），配合物理命中更脆。</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" t="n">
+        <v>2</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="n">
+        <v>1</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>gene_frostfilm</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="n">
+        <v>8132</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>谐振</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>需要器官。改装：命中点按节奏多打几次，打得越散回响越多。</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" t="n">
+        <v>2</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" t="n">
+        <v>1</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0</v>
+      </c>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>gene_harmonic</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="n">
+        <v>8133</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>膜反弹</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>需要器官。改装：撞墙会弹回来，还带一下伤。</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" t="n">
+        <v>2</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0</v>
+      </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>gene_membrane</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="n">
+        <v>8134</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>迟绽</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>需要器官。改装：先飞一会儿，稍后才裂开。</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" t="n">
+        <v>2</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0</v>
+      </c>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>gene_bloomlate</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="n">
+        <v>8135</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>散播</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>需要器官。改装：命中会在旁边炸出小坑。</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Rare</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>2</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>gene_scatterseed</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="n">
+        <v>8136</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>抛投</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>需要器官。改装：攻击像抛物线一样落下。</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" t="n">
+        <v>1</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr"/>
+      <c r="P56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>gene_arc</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="n">
+        <v>8137</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>磁聚</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>需要器官。改装：弹道边飞边被拉向一点。</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" t="n">
+        <v>1</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0</v>
+      </c>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
+      <c r="P57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>gene_magnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="n">
+        <v>8138</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>毛细扩散</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>需要器官。改装：坑/洼会向旁边持续蔓延。</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>2</v>
+      </c>
+      <c r="H58" t="n">
+        <v>1</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" t="n">
+        <v>1</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0</v>
+      </c>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr"/>
+      <c r="P58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>gene_capillary</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="n">
+        <v>8139</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>编织</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>需要器官。改装：把留下的坑/迹跟附近的连起来。</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>2</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="n">
+        <v>1</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0</v>
+      </c>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr"/>
+      <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>gene_weave</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="n">
+        <v>8140</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>催化</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>需要器官。改装：命中触发的 Tag 反应会被放大。</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>2</v>
+      </c>
+      <c r="H60" t="n">
+        <v>1</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>1</v>
+      </c>
+      <c r="K60" t="n">
+        <v>1</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0</v>
+      </c>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr"/>
+      <c r="P60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Gene</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>gene_catalyst</t>
         </is>
       </c>
     </row>

</xml_diff>